<commit_message>
Saved packages open in Office without repair
- jade-opc: a part written into a package with no content type for it — a
  relationships part or a picture added to one that declares every part by
  `Override`, as some decks do — gets a `Default` for its extension when
  the package is written. PowerPoint repaired a deck whose notes jade had
  added (ececapstonespring2012.pptx): the notes' `.rels` had no type.
- jade-xlsx-writer: a sheet whose rows or cells were left out of order by
  another writer is put in order when it is edited. Excel repairs such a
  sheet by dropping its cells.
- The sample, active-sheet and hidden-sheets fixtures had row 7 after
  row 10, which Excel repaired by dropping the sheet's cells; their rows
  are in order now.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/fixtures/active-sheet-workbook.xlsx
+++ b/public/fixtures/active-sheet-workbook.xlsx
@@ -301,6 +301,23 @@
         <v>13535000</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="5">
+        <f>SUM(B4:B6)</f>
+        <v>28400000</v>
+      </c>
+      <c r="C7" s="5">
+        <f>SUM(C4:C6)</f>
+        <v>31625000</v>
+      </c>
+      <c r="D7" s="5">
+        <f>SUM(D4:D6)</f>
+        <v>60025000</v>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" s="3" t="s">
         <v>11</v>
@@ -323,23 +340,6 @@
         <v>10</v>
       </c>
       <c r="D10" s="10"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="5">
-        <f>SUM(B4:B6)</f>
-        <v>28400000</v>
-      </c>
-      <c r="C7" s="5">
-        <f>SUM(C4:C6)</f>
-        <v>31625000</v>
-      </c>
-      <c r="D7" s="5">
-        <f>SUM(D4:D6)</f>
-        <v>60025000</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>